<commit_message>
Update New Station Excel File
</commit_message>
<xml_diff>
--- a/namelist_files_and_local_scripts/time_series_station_files_2_dom_all.xlsx
+++ b/namelist_files_and_local_scripts/time_series_station_files_2_dom_all.xlsx
@@ -1,39 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10312"/>
-  <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wjc/GitHub/SD_Mines_WRF_REALTIME/namelist_files_and_local_scripts/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB828546-685F-BF41-8B27-78B2807CC4CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+  <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="2200" yWindow="1020" windowWidth="30240" windowHeight="17740" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="114">
   <si>
     <t>Station ID</t>
   </si>
@@ -65,6 +46,9 @@
     <t>KUDX</t>
   </si>
   <si>
+    <t>K49B</t>
+  </si>
+  <si>
     <t>KCUT</t>
   </si>
   <si>
@@ -92,15 +76,24 @@
     <t>KD07</t>
   </si>
   <si>
+    <t>K9V6</t>
+  </si>
+  <si>
     <t>KGRN</t>
   </si>
   <si>
     <t>K2WX</t>
   </si>
   <si>
+    <t>K84D</t>
+  </si>
+  <si>
     <t>KGCC</t>
   </si>
   <si>
+    <t>KSUO</t>
+  </si>
+  <si>
     <t>KHEI</t>
   </si>
   <si>
@@ -140,6 +133,18 @@
     <t>KVTN</t>
   </si>
   <si>
+    <t>KMBG</t>
+  </si>
+  <si>
+    <t>K0D8</t>
+  </si>
+  <si>
+    <t>KY27</t>
+  </si>
+  <si>
+    <t>K7L2</t>
+  </si>
+  <si>
     <t>KCYS</t>
   </si>
   <si>
@@ -191,9 +196,6 @@
     <t>KTOP</t>
   </si>
   <si>
-    <t>Row Label</t>
-  </si>
-  <si>
     <t>Rapid City NWS, SD</t>
   </si>
   <si>
@@ -206,6 +208,9 @@
     <t>Rapid City, NEXRAD, SD</t>
   </si>
   <si>
+    <t>Sturgis Airport, SD</t>
+  </si>
+  <si>
     <t>Custer Airport, SD</t>
   </si>
   <si>
@@ -233,15 +238,24 @@
     <t>Faith Airport, SD</t>
   </si>
   <si>
+    <t>Martin Airport, SD</t>
+  </si>
+  <si>
     <t>Gordon Airport, NE</t>
   </si>
   <si>
     <t>Buffalo, SD</t>
   </si>
   <si>
+    <t>Cheyenne Eagle Butte, SD</t>
+  </si>
+  <si>
     <t>Gillette  Airport, WY</t>
   </si>
   <si>
+    <t>Rosebud Sioux Airport, SD</t>
+  </si>
+  <si>
     <t>Hettinger Airport, ND</t>
   </si>
   <si>
@@ -251,7 +265,7 @@
     <t>Lemmon Airport, SD</t>
   </si>
   <si>
-    <t>Converse, CO Airport, WY</t>
+    <t>Converse, Co. Airport, WY</t>
   </si>
   <si>
     <t>Alliance Airport, NE</t>
@@ -281,6 +295,18 @@
     <t>Miller Field Airport, NE</t>
   </si>
   <si>
+    <t>Mobridge Airport, SD</t>
+  </si>
+  <si>
+    <t>Gettysburg Airport, SD</t>
+  </si>
+  <si>
+    <t>Standing Rock Airport, ND</t>
+  </si>
+  <si>
+    <t>Linton Airport, ND</t>
+  </si>
+  <si>
     <t>Cheyenne NWS, WY</t>
   </si>
   <si>
@@ -311,7 +337,7 @@
     <t>Glasgow NWS, MT</t>
   </si>
   <si>
-    <t>Goodland NWS KS</t>
+    <t>Goodland NWS, KS</t>
   </si>
   <si>
     <t>Hastings NWS, NE</t>
@@ -335,20 +361,14 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -359,7 +379,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -367,44 +387,18 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
@@ -692,44 +686,33 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G47"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="2" max="2" width="8.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.1640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.5" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.1640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="18.33203125" bestFit="1" customWidth="1"/>
-  </cols>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:G55"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
-        <v>52</v>
-      </c>
-      <c r="B1" s="1" t="s">
+    <row r="1" spans="1:7">
+      <c r="B1" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E1" s="1" t="s">
+      <c r="C1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A2" s="1">
-        <v>41</v>
+    <row r="2" spans="1:7">
+      <c r="A2">
+        <v>48</v>
       </c>
       <c r="B2" t="s">
         <v>6</v>
@@ -738,21 +721,21 @@
         <v>2</v>
       </c>
       <c r="D2" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="E2">
-        <v>44.072699999999998</v>
+        <v>44.0727</v>
       </c>
       <c r="F2">
         <v>-103.211</v>
       </c>
       <c r="G2">
-        <v>0.43110557303620273</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A3" s="1">
-        <v>34</v>
+        <v>0.4311055730362027</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7">
+      <c r="A3">
+        <v>40</v>
       </c>
       <c r="B3" t="s">
         <v>7</v>
@@ -761,10 +744,10 @@
         <v>2</v>
       </c>
       <c r="D3" t="s">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="E3">
-        <v>44.133000000000003</v>
+        <v>44.133</v>
       </c>
       <c r="F3">
         <v>-103.1</v>
@@ -773,9 +756,9 @@
         <v>10.6829144055438</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A4" s="1">
-        <v>33</v>
+    <row r="4" spans="1:7">
+      <c r="A4">
+        <v>39</v>
       </c>
       <c r="B4" t="s">
         <v>8</v>
@@ -784,21 +767,21 @@
         <v>2</v>
       </c>
       <c r="D4" t="s">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="E4">
-        <v>44.042999999999999</v>
+        <v>44.043</v>
       </c>
       <c r="F4">
         <v>-103.054</v>
       </c>
       <c r="G4">
-        <v>12.697568715776271</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A5" s="1">
-        <v>40</v>
+        <v>12.69756871577627</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7">
+      <c r="A5">
+        <v>47</v>
       </c>
       <c r="B5" t="s">
         <v>9</v>
@@ -807,21 +790,21 @@
         <v>2</v>
       </c>
       <c r="D5" t="s">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="E5">
-        <v>44.133000000000003</v>
+        <v>44.133</v>
       </c>
       <c r="F5">
         <v>-102.833</v>
       </c>
       <c r="G5">
-        <v>30.519656877499319</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A6" s="1">
-        <v>11</v>
+        <v>30.51965687749932</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
+      <c r="A6">
+        <v>2</v>
       </c>
       <c r="B6" t="s">
         <v>10</v>
@@ -830,21 +813,21 @@
         <v>2</v>
       </c>
       <c r="D6" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="E6">
-        <v>43.732999999999997</v>
+        <v>44.4186</v>
       </c>
       <c r="F6">
-        <v>-103.611</v>
+        <v>-103.377</v>
       </c>
       <c r="G6">
-        <v>49.952992671776983</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A7" s="1">
-        <v>37</v>
+        <v>40.55558142954493</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7">
+      <c r="A7">
+        <v>16</v>
       </c>
       <c r="B7" t="s">
         <v>11</v>
@@ -853,21 +836,21 @@
         <v>2</v>
       </c>
       <c r="D7" t="s">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="E7">
-        <v>44.482999999999997</v>
+        <v>43.733</v>
       </c>
       <c r="F7">
-        <v>-103.783</v>
+        <v>-103.611</v>
       </c>
       <c r="G7">
-        <v>64.535897054594059</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A8" s="1">
-        <v>16</v>
+        <v>49.95299267177698</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7">
+      <c r="A8">
+        <v>43</v>
       </c>
       <c r="B8" t="s">
         <v>12</v>
@@ -876,21 +859,21 @@
         <v>2</v>
       </c>
       <c r="D8" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="E8">
-        <v>44.734000000000002</v>
+        <v>44.483</v>
       </c>
       <c r="F8">
-        <v>-103.86199999999999</v>
+        <v>-103.783</v>
       </c>
       <c r="G8">
-        <v>89.899070756525887</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A9" s="1">
-        <v>43</v>
+        <v>64.53589705459406</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7">
+      <c r="A9">
+        <v>21</v>
       </c>
       <c r="B9" t="s">
         <v>13</v>
@@ -899,21 +882,21 @@
         <v>2</v>
       </c>
       <c r="D9" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="E9">
-        <v>44.6629</v>
+        <v>44.734</v>
       </c>
       <c r="F9">
-        <v>-104.568</v>
+        <v>-103.862</v>
       </c>
       <c r="G9">
-        <v>126.4318242195897</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A10" s="1">
-        <v>31</v>
+        <v>89.89907075652589</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7">
+      <c r="A10">
+        <v>50</v>
       </c>
       <c r="B10" t="s">
         <v>14</v>
@@ -922,21 +905,21 @@
         <v>2</v>
       </c>
       <c r="D10" t="s">
-        <v>61</v>
+        <v>68</v>
       </c>
       <c r="E10">
-        <v>44.051000000000002</v>
+        <v>44.6629</v>
       </c>
       <c r="F10">
-        <v>-101.601</v>
+        <v>-104.568</v>
       </c>
       <c r="G10">
-        <v>128.3140564897644</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A11" s="1">
-        <v>26</v>
+        <v>126.4318242195897</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7">
+      <c r="A11">
+        <v>37</v>
       </c>
       <c r="B11" t="s">
         <v>15</v>
@@ -945,21 +928,21 @@
         <v>2</v>
       </c>
       <c r="D11" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="E11">
-        <v>43.021000000000001</v>
+        <v>44.051</v>
       </c>
       <c r="F11">
-        <v>-102.518</v>
+        <v>-101.601</v>
       </c>
       <c r="G11">
-        <v>129.6643847777365</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A12" s="1">
-        <v>10</v>
+        <v>128.3140564897644</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7">
+      <c r="A12">
+        <v>31</v>
       </c>
       <c r="B12" t="s">
         <v>16</v>
@@ -968,21 +951,21 @@
         <v>2</v>
       </c>
       <c r="D12" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="E12">
-        <v>42.837000000000003</v>
+        <v>43.021</v>
       </c>
       <c r="F12">
-        <v>-103.098</v>
+        <v>-102.518</v>
       </c>
       <c r="G12">
-        <v>137.9287007506741</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A13" s="1">
-        <v>2</v>
+        <v>129.6643847777365</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7">
+      <c r="A13">
+        <v>15</v>
       </c>
       <c r="B13" t="s">
         <v>17</v>
@@ -991,21 +974,21 @@
         <v>2</v>
       </c>
       <c r="D13" t="s">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="E13">
-        <v>44.267000000000003</v>
+        <v>42.837</v>
       </c>
       <c r="F13">
-        <v>-104.95</v>
+        <v>-103.098</v>
       </c>
       <c r="G13">
-        <v>140.67735210755981</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A14" s="1">
-        <v>13</v>
+        <v>137.9287007506741</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7">
+      <c r="A14">
+        <v>4</v>
       </c>
       <c r="B14" t="s">
         <v>18</v>
@@ -1014,21 +997,21 @@
         <v>2</v>
       </c>
       <c r="D14" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="E14">
-        <v>45.031999999999996</v>
+        <v>44.267</v>
       </c>
       <c r="F14">
-        <v>-102.01900000000001</v>
+        <v>-104.95</v>
       </c>
       <c r="G14">
-        <v>142.05525337765619</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A15" s="1">
-        <v>24</v>
+        <v>140.6773521075598</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7">
+      <c r="A15">
+        <v>18</v>
       </c>
       <c r="B15" t="s">
         <v>19</v>
@@ -1037,21 +1020,21 @@
         <v>2</v>
       </c>
       <c r="D15" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="E15">
-        <v>42.805999999999997</v>
+        <v>45.032</v>
       </c>
       <c r="F15">
-        <v>-102.175</v>
+        <v>-102.019</v>
       </c>
       <c r="G15">
-        <v>163.84109268787159</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A16" s="1">
-        <v>0</v>
+        <v>142.0552533776562</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7">
+      <c r="A16">
+        <v>7</v>
       </c>
       <c r="B16" t="s">
         <v>20</v>
@@ -1060,21 +1043,21 @@
         <v>2</v>
       </c>
       <c r="D16" t="s">
-        <v>67</v>
+        <v>74</v>
       </c>
       <c r="E16">
-        <v>45.603999999999999</v>
+        <v>43.1656</v>
       </c>
       <c r="F16">
-        <v>-103.54600000000001</v>
+        <v>-101.713</v>
       </c>
       <c r="G16">
-        <v>172.11964229673859</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A17" s="1">
-        <v>19</v>
+        <v>157.0886305290971</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7">
+      <c r="A17">
+        <v>29</v>
       </c>
       <c r="B17" t="s">
         <v>21</v>
@@ -1083,21 +1066,21 @@
         <v>2</v>
       </c>
       <c r="D17" t="s">
-        <v>68</v>
+        <v>75</v>
       </c>
       <c r="E17">
-        <v>44.338999999999999</v>
+        <v>42.806</v>
       </c>
       <c r="F17">
-        <v>-105.542</v>
+        <v>-102.175</v>
       </c>
       <c r="G17">
-        <v>188.4463325816937</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A18" s="1">
-        <v>25</v>
+        <v>163.8410926878716</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7">
+      <c r="A18">
+        <v>1</v>
       </c>
       <c r="B18" t="s">
         <v>22</v>
@@ -1106,21 +1089,21 @@
         <v>2</v>
       </c>
       <c r="D18" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="E18">
-        <v>46.014000000000003</v>
+        <v>45.604</v>
       </c>
       <c r="F18">
-        <v>-102.655</v>
+        <v>-103.546</v>
       </c>
       <c r="G18">
-        <v>219.9266419672897</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A19" s="1">
-        <v>44</v>
+        <v>172.1196422967386</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7">
+      <c r="A19">
+        <v>6</v>
       </c>
       <c r="B19" t="s">
         <v>23</v>
@@ -1129,21 +1112,21 @@
         <v>2</v>
       </c>
       <c r="D19" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="E19">
-        <v>45.933</v>
+        <v>44.9844</v>
       </c>
       <c r="F19">
-        <v>-102.167</v>
+        <v>-101.251</v>
       </c>
       <c r="G19">
-        <v>222.18330501652889</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A20" s="1">
-        <v>28</v>
+        <v>185.0799231815925</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7">
+      <c r="A20">
+        <v>24</v>
       </c>
       <c r="B20" t="s">
         <v>24</v>
@@ -1152,21 +1135,21 @@
         <v>2</v>
       </c>
       <c r="D20" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="E20">
-        <v>45.918999999999997</v>
+        <v>44.339</v>
       </c>
       <c r="F20">
-        <v>-102.10599999999999</v>
+        <v>-105.542</v>
       </c>
       <c r="G20">
-        <v>222.5603248457729</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A21" s="1">
-        <v>15</v>
+        <v>188.4463325816937</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7">
+      <c r="A21">
+        <v>44</v>
       </c>
       <c r="B21" t="s">
         <v>25</v>
@@ -1175,44 +1158,44 @@
         <v>2</v>
       </c>
       <c r="D21" t="s">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="E21">
-        <v>42.795999999999999</v>
+        <v>43.2585</v>
       </c>
       <c r="F21">
-        <v>-105.38</v>
+        <v>-100.859</v>
       </c>
       <c r="G21">
-        <v>225.86355147601409</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A22" s="1">
-        <v>4</v>
+        <v>209.5047045690095</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7">
+      <c r="A22">
+        <v>30</v>
       </c>
       <c r="B22" t="s">
         <v>26</v>
       </c>
       <c r="C22">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D22" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="E22">
-        <v>42.05</v>
+        <v>46.014</v>
       </c>
       <c r="F22">
-        <v>-102.8</v>
+        <v>-102.655</v>
       </c>
       <c r="G22">
-        <v>227.56944345410579</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A23" s="1">
-        <v>1</v>
+        <v>219.9266419672897</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7">
+      <c r="A23">
+        <v>51</v>
       </c>
       <c r="B23" t="s">
         <v>27</v>
@@ -1221,21 +1204,21 @@
         <v>2</v>
       </c>
       <c r="D23" t="s">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="E23">
-        <v>42.75</v>
+        <v>45.933</v>
       </c>
       <c r="F23">
-        <v>-105.383</v>
+        <v>-102.167</v>
       </c>
       <c r="G23">
-        <v>229.35449555827219</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A24" s="1">
-        <v>8</v>
+        <v>222.1833050165289</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7">
+      <c r="A24">
+        <v>33</v>
       </c>
       <c r="B24" t="s">
         <v>28</v>
@@ -1244,90 +1227,90 @@
         <v>2</v>
       </c>
       <c r="D24" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="E24">
-        <v>46.165500000000002</v>
+        <v>45.919</v>
       </c>
       <c r="F24">
-        <v>-103.3</v>
+        <v>-102.106</v>
       </c>
       <c r="G24">
-        <v>232.57826975850921</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A25" s="1">
-        <v>36</v>
+        <v>222.5603248457729</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7">
+      <c r="A25">
+        <v>20</v>
       </c>
       <c r="B25" t="s">
         <v>29</v>
       </c>
       <c r="C25">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D25" t="s">
-        <v>76</v>
+        <v>83</v>
       </c>
       <c r="E25">
-        <v>42.433</v>
+        <v>42.796</v>
       </c>
       <c r="F25">
-        <v>-105.033</v>
+        <v>-105.38</v>
       </c>
       <c r="G25">
-        <v>234.958321162521</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A26" s="1">
-        <v>32</v>
+        <v>225.8635514760141</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7">
+      <c r="A26">
+        <v>9</v>
       </c>
       <c r="B26" t="s">
         <v>30</v>
       </c>
       <c r="C26">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D26" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="E26">
-        <v>44.381</v>
+        <v>42.05</v>
       </c>
       <c r="F26">
-        <v>-100.286</v>
+        <v>-102.8</v>
       </c>
       <c r="G26">
-        <v>235.17103910391759</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A27" s="1">
-        <v>39</v>
+        <v>227.5694434541058</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7">
+      <c r="A27">
+        <v>3</v>
       </c>
       <c r="B27" t="s">
         <v>31</v>
       </c>
       <c r="C27">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D27" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="E27">
-        <v>42.061</v>
+        <v>42.75</v>
       </c>
       <c r="F27">
-        <v>-104.158</v>
+        <v>-105.383</v>
       </c>
       <c r="G27">
-        <v>236.8945391456204</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A28" s="1">
-        <v>29</v>
+        <v>229.3544955582722</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7">
+      <c r="A28">
+        <v>13</v>
       </c>
       <c r="B28" t="s">
         <v>32</v>
@@ -1336,21 +1319,21 @@
         <v>2</v>
       </c>
       <c r="D28" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="E28">
-        <v>43.033000000000001</v>
+        <v>46.1655</v>
       </c>
       <c r="F28">
-        <v>-100.617</v>
+        <v>-103.3</v>
       </c>
       <c r="G28">
-        <v>238.6696483350994</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A29" s="1">
-        <v>5</v>
+        <v>232.5782697585092</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7">
+      <c r="A29">
+        <v>42</v>
       </c>
       <c r="B29" t="s">
         <v>33</v>
@@ -1359,21 +1342,21 @@
         <v>1</v>
       </c>
       <c r="D29" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="E29">
-        <v>41.871000000000002</v>
+        <v>42.433</v>
       </c>
       <c r="F29">
-        <v>-103.593</v>
+        <v>-105.033</v>
       </c>
       <c r="G29">
-        <v>247.07206353589669</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A30" s="1">
-        <v>42</v>
+        <v>234.958321162521</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7">
+      <c r="A30">
+        <v>38</v>
       </c>
       <c r="B30" t="s">
         <v>34</v>
@@ -1382,21 +1365,21 @@
         <v>2</v>
       </c>
       <c r="D30" t="s">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="E30">
-        <v>42.878</v>
+        <v>44.381</v>
       </c>
       <c r="F30">
-        <v>-100.55</v>
+        <v>-100.286</v>
       </c>
       <c r="G30">
-        <v>252.2939738268428</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A31" s="1">
-        <v>12</v>
+        <v>235.1710391039176</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7">
+      <c r="A31">
+        <v>46</v>
       </c>
       <c r="B31" t="s">
         <v>35</v>
@@ -1405,44 +1388,44 @@
         <v>1</v>
       </c>
       <c r="D31" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="E31">
-        <v>41.1556</v>
+        <v>42.061</v>
       </c>
       <c r="F31">
-        <v>-104.81</v>
+        <v>-104.158</v>
       </c>
       <c r="G31">
-        <v>350.10860643832888</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A32" s="1">
-        <v>6</v>
+        <v>236.8945391456204</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7">
+      <c r="A32">
+        <v>35</v>
       </c>
       <c r="B32" t="s">
         <v>36</v>
       </c>
       <c r="C32">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D32" t="s">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="E32">
-        <v>46.7727</v>
+        <v>43.033</v>
       </c>
       <c r="F32">
-        <v>-100.746</v>
+        <v>-100.617</v>
       </c>
       <c r="G32">
-        <v>356.13651415716993</v>
-      </c>
-    </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A33" s="1">
-        <v>27</v>
+        <v>238.6696483350994</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7">
+      <c r="A33">
+        <v>10</v>
       </c>
       <c r="B33" t="s">
         <v>37</v>
@@ -1451,136 +1434,136 @@
         <v>1</v>
       </c>
       <c r="D33" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="E33">
-        <v>41.126199999999997</v>
+        <v>41.871</v>
       </c>
       <c r="F33">
-        <v>-100.684</v>
+        <v>-103.593</v>
       </c>
       <c r="G33">
-        <v>387.42877367270131</v>
-      </c>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A34" s="1">
-        <v>3</v>
+        <v>247.0720635358967</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7">
+      <c r="A34">
+        <v>49</v>
       </c>
       <c r="B34" t="s">
         <v>38</v>
       </c>
       <c r="C34">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D34" t="s">
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="E34">
-        <v>45.4467</v>
+        <v>42.878</v>
       </c>
       <c r="F34">
-        <v>-98.422399999999996</v>
+        <v>-100.55</v>
       </c>
       <c r="G34">
-        <v>407.2835821076373</v>
-      </c>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A35" s="1">
-        <v>35</v>
+        <v>252.2939738268428</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7">
+      <c r="A35">
+        <v>34</v>
       </c>
       <c r="B35" t="s">
         <v>39</v>
       </c>
       <c r="C35">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D35" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="E35">
-        <v>43.0642</v>
+        <v>45.5463</v>
       </c>
       <c r="F35">
-        <v>-108.46</v>
+        <v>-100.406</v>
       </c>
       <c r="G35">
-        <v>437.82235791428252</v>
-      </c>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A36" s="1">
-        <v>9</v>
+        <v>274.8846919264593</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7">
+      <c r="A36">
+        <v>0</v>
       </c>
       <c r="B36" t="s">
         <v>40</v>
       </c>
       <c r="C36">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D36" t="s">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="E36">
-        <v>45.7502</v>
+        <v>44.9866</v>
       </c>
       <c r="F36">
-        <v>-108.57</v>
+        <v>-99.9529</v>
       </c>
       <c r="G36">
-        <v>461.48398607652422</v>
-      </c>
-    </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A37" s="1">
-        <v>14</v>
+        <v>277.0944709174042</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7">
+      <c r="A37">
+        <v>52</v>
       </c>
       <c r="B37" t="s">
         <v>41</v>
       </c>
       <c r="C37">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D37" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="E37">
-        <v>39.861699999999999</v>
+        <v>46.0669</v>
       </c>
       <c r="F37">
-        <v>-104.673</v>
+        <v>-100.633</v>
       </c>
       <c r="G37">
-        <v>483.89787803782338</v>
-      </c>
-    </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A38" s="1">
-        <v>7</v>
+        <v>299.8110310699245</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7">
+      <c r="A38">
+        <v>5</v>
       </c>
       <c r="B38" t="s">
         <v>42</v>
       </c>
       <c r="C38">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D38" t="s">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="E38">
-        <v>39.991999999999997</v>
+        <v>46.2206</v>
       </c>
       <c r="F38">
-        <v>-105.261</v>
+        <v>-100.246</v>
       </c>
       <c r="G38">
-        <v>484.62654498579639</v>
-      </c>
-    </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A39" s="1">
-        <v>18</v>
+        <v>332.8674304096082</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7">
+      <c r="A39">
+        <v>17</v>
       </c>
       <c r="B39" t="s">
         <v>43</v>
@@ -1589,21 +1572,21 @@
         <v>1</v>
       </c>
       <c r="D39" t="s">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="E39">
-        <v>43.582000000000001</v>
+        <v>41.1556</v>
       </c>
       <c r="F39">
-        <v>-96.741900000000001</v>
+        <v>-104.81</v>
       </c>
       <c r="G39">
-        <v>521.33382524072977</v>
-      </c>
-    </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A40" s="1">
-        <v>20</v>
+        <v>350.1086064383289</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7">
+      <c r="A40">
+        <v>11</v>
       </c>
       <c r="B40" t="s">
         <v>44</v>
@@ -1612,21 +1595,21 @@
         <v>1</v>
       </c>
       <c r="D40" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="E40">
-        <v>48.212400000000002</v>
+        <v>46.7727</v>
       </c>
       <c r="F40">
-        <v>-106.61499999999999</v>
+        <v>-100.746</v>
       </c>
       <c r="G40">
-        <v>529.60258153152961</v>
-      </c>
-    </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A41" s="1">
-        <v>23</v>
+        <v>356.1365141571699</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7">
+      <c r="A41">
+        <v>32</v>
       </c>
       <c r="B41" t="s">
         <v>45</v>
@@ -1635,21 +1618,21 @@
         <v>1</v>
       </c>
       <c r="D41" t="s">
-        <v>92</v>
+        <v>99</v>
       </c>
       <c r="E41">
-        <v>39.370699999999999</v>
+        <v>41.1262</v>
       </c>
       <c r="F41">
-        <v>-101.699</v>
+        <v>-100.684</v>
       </c>
       <c r="G41">
-        <v>537.81299158903198</v>
-      </c>
-    </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A42" s="1">
-        <v>21</v>
+        <v>387.4287736727013</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7">
+      <c r="A42">
+        <v>8</v>
       </c>
       <c r="B42" t="s">
         <v>46</v>
@@ -1658,21 +1641,21 @@
         <v>1</v>
       </c>
       <c r="D42" t="s">
-        <v>93</v>
+        <v>100</v>
       </c>
       <c r="E42">
-        <v>40.647500000000001</v>
+        <v>45.4467</v>
       </c>
       <c r="F42">
-        <v>-98.383700000000005</v>
+        <v>-98.4224</v>
       </c>
       <c r="G42">
-        <v>549.60430011219228</v>
-      </c>
-    </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A43" s="1">
-        <v>45</v>
+        <v>407.2835821076373</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7">
+      <c r="A43">
+        <v>41</v>
       </c>
       <c r="B43" t="s">
         <v>47</v>
@@ -1681,21 +1664,21 @@
         <v>1</v>
       </c>
       <c r="D43" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="E43">
-        <v>48.667499999999997</v>
+        <v>43.0642</v>
       </c>
       <c r="F43">
-        <v>-98.834400000000002</v>
+        <v>-108.46</v>
       </c>
       <c r="G43">
-        <v>610.75548649454925</v>
-      </c>
-    </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A44" s="1">
-        <v>17</v>
+        <v>437.8223579142825</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7">
+      <c r="A44">
+        <v>14</v>
       </c>
       <c r="B44" t="s">
         <v>48</v>
@@ -1704,21 +1687,21 @@
         <v>1</v>
       </c>
       <c r="D44" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="E44">
-        <v>47.921900000000001</v>
+        <v>45.7502</v>
       </c>
       <c r="F44">
-        <v>-97.098100000000002</v>
+        <v>-108.57</v>
       </c>
       <c r="G44">
-        <v>636.5233353769745</v>
-      </c>
-    </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A45" s="1">
-        <v>30</v>
+        <v>461.4839860765242</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7">
+      <c r="A45">
+        <v>19</v>
       </c>
       <c r="B45" t="s">
         <v>49</v>
@@ -1727,21 +1710,21 @@
         <v>1</v>
       </c>
       <c r="D45" t="s">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="E45">
-        <v>41.319699999999997</v>
+        <v>39.8617</v>
       </c>
       <c r="F45">
-        <v>-96.367000000000004</v>
+        <v>-104.673</v>
       </c>
       <c r="G45">
-        <v>637.10022550210772</v>
-      </c>
-    </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A46" s="1">
-        <v>22</v>
+        <v>483.8978780378234</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7">
+      <c r="A46">
+        <v>12</v>
       </c>
       <c r="B46" t="s">
         <v>50</v>
@@ -1750,21 +1733,21 @@
         <v>1</v>
       </c>
       <c r="D46" t="s">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="E46">
-        <v>39.122399999999999</v>
+        <v>39.992</v>
       </c>
       <c r="F46">
-        <v>-108.527</v>
+        <v>-105.261</v>
       </c>
       <c r="G46">
-        <v>706.05970680141979</v>
-      </c>
-    </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A47" s="1">
-        <v>38</v>
+        <v>484.6265449857964</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7">
+      <c r="A47">
+        <v>23</v>
       </c>
       <c r="B47" t="s">
         <v>51</v>
@@ -1773,19 +1756,203 @@
         <v>1</v>
       </c>
       <c r="D47" t="s">
-        <v>98</v>
+        <v>105</v>
       </c>
       <c r="E47">
-        <v>39.068800000000003</v>
+        <v>43.582</v>
       </c>
       <c r="F47">
-        <v>-95.622399999999999</v>
+        <v>-96.7419</v>
       </c>
       <c r="G47">
-        <v>840.71703075227481</v>
+        <v>521.3338252407298</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7">
+      <c r="A48">
+        <v>25</v>
+      </c>
+      <c r="B48" t="s">
+        <v>52</v>
+      </c>
+      <c r="C48">
+        <v>1</v>
+      </c>
+      <c r="D48" t="s">
+        <v>106</v>
+      </c>
+      <c r="E48">
+        <v>48.2124</v>
+      </c>
+      <c r="F48">
+        <v>-106.615</v>
+      </c>
+      <c r="G48">
+        <v>529.6025815315296</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7">
+      <c r="A49">
+        <v>28</v>
+      </c>
+      <c r="B49" t="s">
+        <v>53</v>
+      </c>
+      <c r="C49">
+        <v>1</v>
+      </c>
+      <c r="D49" t="s">
+        <v>107</v>
+      </c>
+      <c r="E49">
+        <v>39.3707</v>
+      </c>
+      <c r="F49">
+        <v>-101.699</v>
+      </c>
+      <c r="G49">
+        <v>537.812991589032</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7">
+      <c r="A50">
+        <v>26</v>
+      </c>
+      <c r="B50" t="s">
+        <v>54</v>
+      </c>
+      <c r="C50">
+        <v>1</v>
+      </c>
+      <c r="D50" t="s">
+        <v>108</v>
+      </c>
+      <c r="E50">
+        <v>40.6475</v>
+      </c>
+      <c r="F50">
+        <v>-98.3837</v>
+      </c>
+      <c r="G50">
+        <v>549.6043001121923</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7">
+      <c r="A51">
+        <v>53</v>
+      </c>
+      <c r="B51" t="s">
+        <v>55</v>
+      </c>
+      <c r="C51">
+        <v>1</v>
+      </c>
+      <c r="D51" t="s">
+        <v>109</v>
+      </c>
+      <c r="E51">
+        <v>48.6675</v>
+      </c>
+      <c r="F51">
+        <v>-98.8344</v>
+      </c>
+      <c r="G51">
+        <v>610.7554864945492</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7">
+      <c r="A52">
+        <v>22</v>
+      </c>
+      <c r="B52" t="s">
+        <v>56</v>
+      </c>
+      <c r="C52">
+        <v>1</v>
+      </c>
+      <c r="D52" t="s">
+        <v>110</v>
+      </c>
+      <c r="E52">
+        <v>47.9219</v>
+      </c>
+      <c r="F52">
+        <v>-97.0981</v>
+      </c>
+      <c r="G52">
+        <v>636.5233353769745</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7">
+      <c r="A53">
+        <v>36</v>
+      </c>
+      <c r="B53" t="s">
+        <v>57</v>
+      </c>
+      <c r="C53">
+        <v>1</v>
+      </c>
+      <c r="D53" t="s">
+        <v>111</v>
+      </c>
+      <c r="E53">
+        <v>41.3197</v>
+      </c>
+      <c r="F53">
+        <v>-96.3673</v>
+      </c>
+      <c r="G53">
+        <v>637.0787546201985</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7">
+      <c r="A54">
+        <v>27</v>
+      </c>
+      <c r="B54" t="s">
+        <v>58</v>
+      </c>
+      <c r="C54">
+        <v>1</v>
+      </c>
+      <c r="D54" t="s">
+        <v>112</v>
+      </c>
+      <c r="E54">
+        <v>39.1224</v>
+      </c>
+      <c r="F54">
+        <v>-108.527</v>
+      </c>
+      <c r="G54">
+        <v>706.0597068014198</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7">
+      <c r="A55">
+        <v>45</v>
+      </c>
+      <c r="B55" t="s">
+        <v>59</v>
+      </c>
+      <c r="C55">
+        <v>1</v>
+      </c>
+      <c r="D55" t="s">
+        <v>113</v>
+      </c>
+      <c r="E55">
+        <v>39.0688</v>
+      </c>
+      <c r="F55">
+        <v>-95.6224</v>
+      </c>
+      <c r="G55">
+        <v>840.7170307522748</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Adding Huron to Station List
</commit_message>
<xml_diff>
--- a/namelist_files_and_local_scripts/time_series_station_files_2_dom_all.xlsx
+++ b/namelist_files_and_local_scripts/time_series_station_files_2_dom_all.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10713"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10719"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wjc/GitHub/SD_Mines_WRF_REALTIME/namelist_files_and_local_scripts/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{524DC369-2BED-A34D-9450-C43B8BDCF725}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B258A56A-6666-2E47-8C50-33263153DF06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>

</xml_diff>